<commit_message>
chore: bump to 1.1.6 + changelog
1.1.5 is already approved and live, which closes its train:

  ITMS-90186: The train version '1.1.5' is closed for new build submissions
  ITMS-90062: CFBundleShortVersionString [1.1.5] must contain a higher
              version than the previously approved version [1.1.5]

That, not a duplicate build number, is what rejected builds 67/89/91/95.
Every upload was going to an already-approved version.

Bumped app.json, package.json and MARKETING_VERSION. Info.plist now
derives from $(MARKETING_VERSION) after a988d5e, so it is no longer a
fourth place to miss.

Changelog updated in the same commit per CLAUDE.md, with 14 rows for
today. 1.1.6 registered in the Summary sheet's release list so the rows
are actually counted.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-07-29.</t>
+          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-08-16.</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E79)</f>
+        <f>COUNTA(Changes!E2:E93)</f>
         <v/>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$79,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$93,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$79,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$93,G8)</f>
         <v/>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$79,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$93,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$79,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$93,G9)</f>
         <v/>
       </c>
     </row>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$79,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$93,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$79,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$93,G10)</f>
         <v/>
       </c>
     </row>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$79,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$93,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -753,16 +753,16 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Unreleased</t>
+          <t>1.1.6</t>
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$79,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$93,G11)</f>
         <v/>
       </c>
     </row>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$79,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$93,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -782,7 +782,16 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H12" s="7">
+        <f>COUNTIF(Changes!$G$2:$G$93,G12)</f>
         <v/>
       </c>
     </row>
@@ -793,7 +802,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$79,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$93,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -802,7 +811,7 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D13)</f>
         <v/>
       </c>
     </row>
@@ -813,7 +822,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$79,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$93,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -822,7 +831,7 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D14)</f>
         <v/>
       </c>
     </row>
@@ -833,7 +842,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D15)</f>
         <v/>
       </c>
     </row>
@@ -844,7 +853,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D16)</f>
         <v/>
       </c>
     </row>
@@ -855,7 +864,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D17)</f>
         <v/>
       </c>
     </row>
@@ -866,7 +875,7 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D18)</f>
         <v/>
       </c>
     </row>
@@ -877,7 +886,7 @@
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D19)</f>
         <v/>
       </c>
     </row>
@@ -888,194 +897,238 @@
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Interaction</t>
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Scaling</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Screen Time</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Scaling</t>
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Tasks</t>
+          <t>Screen Time</t>
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Tour</t>
+          <t>Siri</t>
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$93,D33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="D34" s="7" t="inlineStr">
         <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="E34" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$93,D34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="E35" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$93,D35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Tour</t>
+        </is>
+      </c>
+      <c r="E36" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$93,D36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="D37" s="7" t="inlineStr">
+        <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$79,D34)</f>
+      <c r="E37" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$93,D37)</f>
         <v/>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="38">
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="E38" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$93,D38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>• 1.1.4 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>• Counts on this sheet are formulas over the Changes tab — they update if you edit, add or delete rows there.</t>
         </is>
@@ -1092,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4415,8 +4468,596 @@
         </is>
       </c>
     </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>788c3c0</t>
+        </is>
+      </c>
+      <c r="C80" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D80" s="15" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="E80" s="18" t="inlineStr">
+        <is>
+          <t>Calendar-imported tasks skipped AI verification entirely</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="inlineStr">
+        <is>
+          <t>Tasks created from the calendar suggestion sheet were hardcoded aiCheck: false, so tapping one claimed the credit instantly while every manually-created task went through the AI proof check. Now inherits proAccess like any other task.</t>
+        </is>
+      </c>
+      <c r="G80" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H80" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B81" s="16" t="inlineStr">
+        <is>
+          <t>788c3c0</t>
+        </is>
+      </c>
+      <c r="C81" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="E81" s="18" t="inlineStr">
+        <is>
+          <t>Users signed out at random, not just after updates</t>
+        </is>
+      </c>
+      <c r="F81" s="18" t="inlineStr">
+        <is>
+          <t>safeGetSession called supabase.auth.signOut() whenever an error message matched /invalid.*refresh|refresh.*expired/i. A transient 5xx, or a cold start before the network was ready, matched that regex and destroyed the session before autoRefreshToken could retry. Supabase already emits SIGNED_OUT on a genuinely dead token, so the manual sign-out was both redundant and destructive. NOTE: a second suspected cause (loss of the Keychain AES key, which makes the encrypted session decrypt to garbage) is untouched and still live.</t>
+        </is>
+      </c>
+      <c r="G81" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H81" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>20020dc</t>
+        </is>
+      </c>
+      <c r="C82" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Share-a-win sheet after completing a task</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="inlineStr">
+        <is>
+          <t>Every third task completed in a day offers a share sheet with the task, duration and time earned, plus an App Store link. Built on React Native's built-in Share, so no new dependency.</t>
+        </is>
+      </c>
+      <c r="G82" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H82" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="40" customHeight="1">
+      <c r="A83" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B83" s="16" t="inlineStr">
+        <is>
+          <t>be399eb</t>
+        </is>
+      </c>
+      <c r="C83" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
+        <is>
+          <t>Siri</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Four Siri voice commands via App Intents</t>
+        </is>
+      </c>
+      <c r="F83" s="18" t="inlineStr">
+        <is>
+          <t>Check balance, create task, start a Drift In session, and today's progress. Registered through AppShortcutsProvider so they also surface in Shortcuts. App Intents needs no entitlement and no App Store Connect configuration, unlike the deprecated SiriKit.</t>
+        </is>
+      </c>
+      <c r="G83" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H83" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="40" customHeight="1">
+      <c r="A84" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>4fba037</t>
+        </is>
+      </c>
+      <c r="C84" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Onboarding slide introducing the Siri commands</t>
+        </is>
+      </c>
+      <c r="F84" s="18" t="inlineStr">
+        <is>
+          <t>Fifth how-it-works slide listing the three main utterances, so the feature is discoverable rather than hidden.</t>
+        </is>
+      </c>
+      <c r="G84" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H84" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="40" customHeight="1">
+      <c r="A85" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B85" s="16" t="inlineStr">
+        <is>
+          <t>4fba037</t>
+        </is>
+      </c>
+      <c r="C85" s="23" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="E85" s="18" t="inlineStr">
+        <is>
+          <t>Buttons now give haptic feedback on press</t>
+        </is>
+      </c>
+      <c r="F85" s="18" t="inlineStr">
+        <is>
+          <t>Anim.Pop accepted a `haptic` prop and silently ignored it - expo-haptics was installed but never reached the button layer. Now fires on press-in rather than onPress, so the tick lands at contact instead of reading as lag. Opt-in per call site.</t>
+        </is>
+      </c>
+      <c r="G85" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H85" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="40" customHeight="1">
+      <c r="A86" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B86" s="16" t="inlineStr">
+        <is>
+          <t>4fba037</t>
+        </is>
+      </c>
+      <c r="C86" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D86" s="15" t="inlineStr">
+        <is>
+          <t>Screen Time</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Mid-session nudge while burning earned time</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="inlineStr">
+        <is>
+          <t>A silent notification (Is this really the move right now?) fires from the DeviceActivity checkpoint, capped at 4 per day. That checkpoint is the only moment iOS tells a third-party app the user is mid-session on a blocked app.</t>
+        </is>
+      </c>
+      <c r="G86" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H86" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="40" customHeight="1">
+      <c r="A87" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B87" s="16" t="inlineStr">
+        <is>
+          <t>9452c72</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
+        <is>
+          <t>Screen Time</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Checkpoint cadence tightened to 5 minutes, with a hard event cap</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="inlineStr">
+        <is>
+          <t>More checkpoints means more chances to nudge. Apple documents a ~15-minute floor for threshold delivery, but whether it applies to event thresholds is unverified; every 15-minute mark is still a multiple of 5, so the worst case degrades to the previous behaviour. Also a safety fix: an 8-hour balance previously armed 31 events, and if startMonitoring throws, the catch stops ALL monitoring and leaves no enforcement at all. Now capped at 17.</t>
+        </is>
+      </c>
+      <c r="G87" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H87" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B88" s="16" t="inlineStr">
+        <is>
+          <t>dbd0fe1</t>
+        </is>
+      </c>
+      <c r="C88" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D88" s="15" t="inlineStr">
+        <is>
+          <t>Screen Time</t>
+        </is>
+      </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Block screen names the app it is blocking</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="inlineStr">
+        <is>
+          <t>ShieldConfigurationDataSource is the one place iOS hands a third-party app the identity of the app being opened, and the parameter was being discarded. The shield can now say Is Instagram the move right now? The name is used only to draw that screen - the extension is sandboxed specifically to prevent moving content out, so it is never persisted or transmitted.</t>
+        </is>
+      </c>
+      <c r="G88" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H88" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="40" customHeight="1">
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B89" s="16" t="inlineStr">
+        <is>
+          <t>a988d5e</t>
+        </is>
+      </c>
+      <c r="C89" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D89" s="15" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Xcode Cloud could not upload builds - versions hardcoded in Info.plist</t>
+        </is>
+      </c>
+      <c r="F89" s="18" t="inlineStr">
+        <is>
+          <t>ios/Drift/Info.plist pinned CFBundleShortVersionString and CFBundleVersion to literals. Info.plist OVERRIDES the build settings, so Xcode Cloud's auto-incremented build number never reached the binary. The three extensions never hit this because their Info.plists do not declare these keys. Now reads $(MARKETING_VERSION) / $(CURRENT_PROJECT_VERSION), which also removes Info.plist as a fourth place every version bump had to be applied.</t>
+        </is>
+      </c>
+      <c r="G89" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H89" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="40" customHeight="1">
+      <c r="A90" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>a4c6895</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D90" s="15" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="inlineStr">
+        <is>
+          <t>Archive failed - every App Shortcut utterance needs the applicationName token</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="inlineStr">
+        <is>
+          <t>Apple rejects the build if any utterance omits it. One of thirteen phrases hardcoded Start Drift In. Since the display name is Drift the token renders inline, so the advertised phrasing was preserved.</t>
+        </is>
+      </c>
+      <c r="G90" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H90" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="40" customHeight="1">
+      <c r="A91" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B91" s="16" t="inlineStr">
+        <is>
+          <t>7b188c2</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D91" s="15" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E91" s="18" t="inlineStr">
+        <is>
+          <t>ci_post_clone no longer fails when Node is already installed</t>
+        </is>
+      </c>
+      <c r="F91" s="18" t="inlineStr">
+        <is>
+          <t>brew install node exits non-zero when the formula is already present, and set -e turned that into a dead build before anything compiled. Newer Xcode Cloud images ship Node, so this fired intermittently depending on which image the build landed on.</t>
+        </is>
+      </c>
+      <c r="G91" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H91" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B92" s="16" t="inlineStr">
+        <is>
+          <t>2c2ced7</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D92" s="15" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="E92" s="18" t="inlineStr">
+        <is>
+          <t>Download links on the marketing site were dead</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="inlineStr">
+        <is>
+          <t>Two different App Store IDs were in circulation across docs/ (6738963592 and 6746262733) and both 404'd. The correct ID is 6778215875, verified against the real bundle id com.sanghani.drift via the iTunes lookup API. The same audit is still outstanding on driftproductivity.com, which is a separate codebase.</t>
+        </is>
+      </c>
+      <c r="G92" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H92" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="40" customHeight="1">
+      <c r="A93" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>2c2ced7</t>
+        </is>
+      </c>
+      <c r="C93" s="21" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D93" s="15" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Blog section, AI and Siri articles, sitemap and structured data</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="inlineStr">
+        <is>
+          <t>Adds a blog index plus posts on AI verification and Siri control, a sitemap.xml and robots.txt (neither existed before), and JSON-LD MobileApplication/Article/FAQPage markup. Published to the GitHub Pages site, NOT to driftproductivity.com - see SITEBLOG.md for that handoff.</t>
+        </is>
+      </c>
+      <c r="G93" s="16" t="inlineStr">
+        <is>
+          <t>1.1.6</t>
+        </is>
+      </c>
+      <c r="H93" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H79"/>
+  <autoFilter ref="A1:H93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: changelog rows for the AI Check outage
Three rows for 0d07a1a: the four-day 400 (root cause: taskId made
mandatory server-side while the client that sends it was still
unreleased), the client-side error-body bug that made it unreadable, and
the undeployed verify-task work the redeploy swept up.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$96</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-08-16.</t>
+          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-08-24.</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E93)</f>
+        <f>COUNTA(Changes!E2:E96)</f>
         <v/>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$93,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$96,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$93,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$96,G8)</f>
         <v/>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$93,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$96,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$93,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$96,G9)</f>
         <v/>
       </c>
     </row>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$93,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$96,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$93,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$96,G10)</f>
         <v/>
       </c>
     </row>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$93,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$96,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$93,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$96,G11)</f>
         <v/>
       </c>
     </row>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$93,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$96,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$93,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$96,G12)</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$93,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$96,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D13)</f>
         <v/>
       </c>
     </row>
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$93,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$96,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D14)</f>
         <v/>
       </c>
     </row>
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D15)</f>
         <v/>
       </c>
     </row>
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D16)</f>
         <v/>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D17)</f>
         <v/>
       </c>
     </row>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D18)</f>
         <v/>
       </c>
     </row>
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D19)</f>
         <v/>
       </c>
     </row>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D20)</f>
         <v/>
       </c>
     </row>
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D21)</f>
         <v/>
       </c>
     </row>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D22)</f>
         <v/>
       </c>
     </row>
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D23)</f>
         <v/>
       </c>
     </row>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D24)</f>
         <v/>
       </c>
     </row>
@@ -952,7 +952,7 @@
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D25)</f>
         <v/>
       </c>
     </row>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D26)</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D27)</f>
         <v/>
       </c>
     </row>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D28)</f>
         <v/>
       </c>
     </row>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D29)</f>
         <v/>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D30)</f>
         <v/>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D31)</f>
         <v/>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D32)</f>
         <v/>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D33)</f>
         <v/>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D34)</f>
         <v/>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D35)</f>
         <v/>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D36)</f>
         <v/>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D37)</f>
         <v/>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$93,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$96,D38)</f>
         <v/>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5056,8 +5056,134 @@
         </is>
       </c>
     </row>
+    <row r="94" ht="40" customHeight="1">
+      <c r="A94" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B94" s="16" t="inlineStr">
+        <is>
+          <t>0d07a1a</t>
+        </is>
+      </c>
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
+        <is>
+          <t>AI Check</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>AI Check was rejecting every submission from every live user</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>verify-task was redeployed on 2026-08-20 making taskId mandatory with a deliberate no-fallback policy, but the client change that sends taskId never shipped - the build in users' hands is 65, which still sends only taskTitle/durationMins. Every submission returned task_id_required (400) for four days. An old client naming a task by TITLE now gets the row looked up instead: the lookup runs through the caller's own RLS-scoped client and returns a real row, so created_at, minutes and the attempt count still come from the database and the time gate still holds - the title only chooses WHICH of the caller's own rows is being checked. user_id is pinned explicitly because the 'tasks: parent select' policy would otherwise let a parent's submission resolve onto a child's identically-named task. Temporary: delete once the taskId-sending build is the minimum supported version.</t>
+        </is>
+      </c>
+      <c r="G94" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H94" s="22" t="inlineStr">
+        <is>
+          <t>Edge deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="40" customHeight="1">
+      <c r="A95" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B95" s="16" t="inlineStr">
+        <is>
+          <t>0d07a1a</t>
+        </is>
+      </c>
+      <c r="C95" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D95" s="15" t="inlineStr">
+        <is>
+          <t>AI Check</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Server error messages never reached the user - everything read as a bare status code</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="inlineStr">
+        <is>
+          <t>The client looked for the error body at res.error.context.response. In functions-js error.context IS the Response; there is no .response wrapper, so body stayed null and every status under 500 fell through to a generic 'the AI service rejected the request (error N)' alert. That is why a four-day outage surfaced as an unexplained 400 instead of the server's own 'Update Drift'. The 402 paywall, 425 too-early, follow-up-question and ai_error branches all read body, so they were silently dead too.</t>
+        </is>
+      </c>
+      <c r="G95" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H95" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="40" customHeight="1">
+      <c r="A96" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B96" s="16" t="inlineStr">
+        <is>
+          <t>0d07a1a</t>
+        </is>
+      </c>
+      <c r="C96" s="20" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>AI Check</t>
+        </is>
+      </c>
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Three commits of undeployed verify-task work went live</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="inlineStr">
+        <is>
+          <t>The deployed function was pinned at the 2026-08-20 16:18 build, predating retroactive-task support and the ask-a-clarifying-question-before-rejecting flow. Caught by diffing the downloaded artifact against the repo - worth doing routinely, since nothing in the deploy path reports drift.</t>
+        </is>
+      </c>
+      <c r="G96" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H96" s="22" t="inlineStr">
+        <is>
+          <t>Edge deploy</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H93"/>
+  <autoFilter ref="A1:H96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: changelog row for the 425 time-gate regression
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E96)</f>
+        <f>COUNTA(Changes!E2:E97)</f>
         <v/>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$96,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$97,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$96,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$97,G8)</f>
         <v/>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$96,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$97,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$96,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$97,G9)</f>
         <v/>
       </c>
     </row>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$96,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$97,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$96,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$97,G10)</f>
         <v/>
       </c>
     </row>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$96,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$97,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$96,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$97,G11)</f>
         <v/>
       </c>
     </row>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$96,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$97,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$96,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$97,G12)</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$96,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$97,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D13)</f>
         <v/>
       </c>
     </row>
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$96,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$97,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D14)</f>
         <v/>
       </c>
     </row>
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D15)</f>
         <v/>
       </c>
     </row>
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D16)</f>
         <v/>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D17)</f>
         <v/>
       </c>
     </row>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D18)</f>
         <v/>
       </c>
     </row>
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D19)</f>
         <v/>
       </c>
     </row>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D20)</f>
         <v/>
       </c>
     </row>
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D21)</f>
         <v/>
       </c>
     </row>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D22)</f>
         <v/>
       </c>
     </row>
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D23)</f>
         <v/>
       </c>
     </row>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D24)</f>
         <v/>
       </c>
     </row>
@@ -952,7 +952,7 @@
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D25)</f>
         <v/>
       </c>
     </row>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D26)</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D27)</f>
         <v/>
       </c>
     </row>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D28)</f>
         <v/>
       </c>
     </row>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D29)</f>
         <v/>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D30)</f>
         <v/>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D31)</f>
         <v/>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D32)</f>
         <v/>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D33)</f>
         <v/>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D34)</f>
         <v/>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D35)</f>
         <v/>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D36)</f>
         <v/>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D37)</f>
         <v/>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$96,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$97,D38)</f>
         <v/>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5182,8 +5182,50 @@
         </is>
       </c>
     </row>
+    <row r="97" ht="40" customHeight="1">
+      <c r="A97" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B97" s="16" t="inlineStr">
+        <is>
+          <t>ac41f39</t>
+        </is>
+      </c>
+      <c r="C97" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D97" s="15" t="inlineStr">
+        <is>
+          <t>AI Check</t>
+        </is>
+      </c>
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Time gate fired as an unexplained error on the shipped build</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="inlineStr">
+        <is>
+          <t>The gate (no proof until half the task duration has elapsed) is server-only behaviour that has never shipped in a client. Build 65 has no countdown, no 'unlocks in 30 min' copy and no branch for 425 - it reads only 402 and 429 by status - so a 60-minute task had a 30-minute window where AI Check just errored with no visible reason. The gate now applies only to clients that send a taskId, which are exactly the clients that can render the countdown and the reason. Same class of mistake as the 400 above: a rule enforced server-side that the client in users' hands cannot express.</t>
+        </is>
+      </c>
+      <c r="G97" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H97" s="22" t="inlineStr">
+        <is>
+          <t>Edge deploy</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H96"/>
+  <autoFilter ref="A1:H97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: changelog row for the duplicate-title selection fix
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E97)</f>
+        <f>COUNTA(Changes!E2:E98)</f>
         <v/>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$97,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$98,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$97,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$98,G8)</f>
         <v/>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$97,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$98,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$97,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$98,G9)</f>
         <v/>
       </c>
     </row>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$97,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$98,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$97,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$98,G10)</f>
         <v/>
       </c>
     </row>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$97,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$98,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$97,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$98,G11)</f>
         <v/>
       </c>
     </row>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$97,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$98,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$97,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$98,G12)</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$97,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$98,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D13)</f>
         <v/>
       </c>
     </row>
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$97,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$98,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D14)</f>
         <v/>
       </c>
     </row>
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D15)</f>
         <v/>
       </c>
     </row>
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D16)</f>
         <v/>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D17)</f>
         <v/>
       </c>
     </row>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D18)</f>
         <v/>
       </c>
     </row>
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D19)</f>
         <v/>
       </c>
     </row>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D20)</f>
         <v/>
       </c>
     </row>
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D21)</f>
         <v/>
       </c>
     </row>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D22)</f>
         <v/>
       </c>
     </row>
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D23)</f>
         <v/>
       </c>
     </row>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D24)</f>
         <v/>
       </c>
     </row>
@@ -952,7 +952,7 @@
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D25)</f>
         <v/>
       </c>
     </row>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D26)</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D27)</f>
         <v/>
       </c>
     </row>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D28)</f>
         <v/>
       </c>
     </row>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D29)</f>
         <v/>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D30)</f>
         <v/>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D31)</f>
         <v/>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D32)</f>
         <v/>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D33)</f>
         <v/>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D34)</f>
         <v/>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D35)</f>
         <v/>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D36)</f>
         <v/>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D37)</f>
         <v/>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$97,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$98,D38)</f>
         <v/>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5224,8 +5224,50 @@
         </is>
       </c>
     </row>
+    <row r="98" ht="40" customHeight="1">
+      <c r="A98" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B98" s="16" t="inlineStr">
+        <is>
+          <t>2282249</t>
+        </is>
+      </c>
+      <c r="C98" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="inlineStr">
+        <is>
+          <t>AI Check</t>
+        </is>
+      </c>
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>Legacy title lookup could block a task the user had never verified</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="inlineStr">
+        <is>
+          <t>The compat path resolves a task by title, and same-title duplicates turn out to be the norm rather than an exception - production carries up to 23 unfinished rows under one title, spanning 19 days, because people re-add 'Make Bed' every morning. Newest-first lands on today's instance correctly, but the client marks ITS row done locally rather than whichever row the server stamped, so two same-titled tasks added on one day could diverge and the next honest submission would come back 'already verified'. Selection now prefers a row that is neither done nor already stamped. Replay protection is unaffected: when the replayed row is the only candidate it is still the one picked. A failed lookup now returns 503 rather than 404, which had been telling users to refresh a list that was fine.</t>
+        </is>
+      </c>
+      <c r="G98" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H98" s="22" t="inlineStr">
+        <is>
+          <t>Edge deploy</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H97"/>
+  <autoFilter ref="A1:H98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(release): build 122 for the 1.1.7 submission, changelog updated
Bumped CURRENT_PROJECT_VERSION 121 -> 122. 121 may already have been consumed
by an upload and a duplicate version+build pair is the ITMS-90062 rejection
that cost builds 56/60/63/64/67/89; a spare build number costs nothing.
MARKETING_VERSION, app.json and package.json are all 1.1.7 and stay put, and
Info.plist keeps both keys variable-driven.

Changelog gains the three 1.1.7 rows this session produced that were not yet
logged: the RevenueCat key mismatch, the NFC sheet copy, and the bedtime
moment. Per CLAUDE.md this belongs in the same commit as the bump.

Verified with a Release build against the iOS 27 SDK: BUILD SUCCEEDED.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-08-27.</t>
+          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-08-28.</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E109)</f>
+        <f>COUNTA(Changes!E2:E112)</f>
         <v/>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$109,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$112,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$109,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$112,G8)</f>
         <v/>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$109,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$112,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$109,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$112,G9)</f>
         <v/>
       </c>
     </row>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$109,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$112,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$109,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$112,G10)</f>
         <v/>
       </c>
     </row>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$109,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$112,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$109,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$112,G11)</f>
         <v/>
       </c>
     </row>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$109,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$112,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$109,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$112,G12)</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$109,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$112,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D13)</f>
         <v/>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="H13" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$109,G13)</f>
+        <f>COUNTIF(Changes!$G$2:$G$112,G13)</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$109,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$112,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -840,7 +840,7 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D14)</f>
         <v/>
       </c>
     </row>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D15)</f>
         <v/>
       </c>
     </row>
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D16)</f>
         <v/>
       </c>
     </row>
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D17)</f>
         <v/>
       </c>
     </row>
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D18)</f>
         <v/>
       </c>
     </row>
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D19)</f>
         <v/>
       </c>
     </row>
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D20)</f>
         <v/>
       </c>
     </row>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D21)</f>
         <v/>
       </c>
     </row>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D22)</f>
         <v/>
       </c>
     </row>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D23)</f>
         <v/>
       </c>
     </row>
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D24)</f>
         <v/>
       </c>
     </row>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D25)</f>
         <v/>
       </c>
     </row>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D26)</f>
         <v/>
       </c>
     </row>
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D27)</f>
         <v/>
       </c>
     </row>
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D28)</f>
         <v/>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D29)</f>
         <v/>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D30)</f>
         <v/>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D31)</f>
         <v/>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D32)</f>
         <v/>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D33)</f>
         <v/>
       </c>
     </row>
@@ -1060,95 +1060,106 @@
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Tasks</t>
+          <t>Sleep Guard</t>
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Tasks</t>
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Tour</t>
+          <t>Theme</t>
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Tour</t>
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$112,D38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="D39" s="7" t="inlineStr">
         <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E39" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$112,D39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="D40" s="7" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="E39" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$109,D39)</f>
+      <c r="E40" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$112,D40)</f>
         <v/>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>• 1.1.4 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
+          <t>• 1.1.4 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
+          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>• Counts on this sheet are formulas over the Changes tab — they update if you edit, add or delete rows there.</t>
         </is>
@@ -1165,7 +1176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5748,8 +5759,134 @@
         </is>
       </c>
     </row>
+    <row r="110" ht="40" customHeight="1">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B110" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C110" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D110" s="15" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Nobody could ever subscribe - the app shipped a RevenueCat key for a different app</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="inlineStr">
+        <is>
+          <t>Purchases.configure() was called with appl_OetkgVkCSGdSfmrXdrqCElOjgIs, which is not the public key for com.sanghani.drift; the dashboard's key is appl_kjgnLRndYGRvEpkIetTELaBUTVZ. The value came from a fallback in useSubscription.js and .env sets no EXPO_PUBLIC_RC_IOS_KEY, so the stale key is what every build has shipped since launch - including 1.1.6, live on the App Store. The SDK identified Drift as another app, so getOfferings() always returned "none of the products registered in the RevenueCat dashboard could be fetched" and every purchase attempt failed with no_offering. It went unnoticed because PaywallScreen falls back to hardcoded $4.99/$29.99 prices when offerings are missing, so the paywall looked healthy while the revenue path was dead. The catalogue itself was fine all along: 7 products on the `pro` entitlement in the `default` offering, with com.drift.pro.month and com.drift.pro.annual already Approved. Purchases still require the Paid Apps Agreement to leave Pending User Info - it has no bank account on file, so Apple serves no products regardless.</t>
+        </is>
+      </c>
+      <c r="G110" s="16" t="inlineStr">
+        <is>
+          <t>1.1.7</t>
+        </is>
+      </c>
+      <c r="H110" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="40" customHeight="1">
+      <c r="A111" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B111" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C111" s="23" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D111" s="15" t="inlineStr">
+        <is>
+          <t>Sleep Guard</t>
+        </is>
+      </c>
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>NFC sheet says what the tap is for, and rejects a wrong tag on the sheet itself</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="inlineStr">
+        <is>
+          <t>iOS renders the NFC sheet and exposes only two strings plus an error line, and both flows shared one hardcoded prompt. It was wrong for registration: a first-time user was told to hold their phone near "the Drift tag" when nothing had been shipped to them - they were designating a blank sticker, and the copy read like a missing package. Registration now says "the tag you want to use", arming says "your tag to start the night" and confirms with "Night started. Your apps are locked until morning." scanTag also takes an expected UID, so arming with the wrong tag fails on the sheet in red instead of showing a green check and contradicting it with an alert a moment later.</t>
+        </is>
+      </c>
+      <c r="G111" s="16" t="inlineStr">
+        <is>
+          <t>1.1.7</t>
+        </is>
+      </c>
+      <c r="H111" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="40" customHeight="1">
+      <c r="A112" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B112" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C112" s="23" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D112" s="15" t="inlineStr">
+        <is>
+          <t>Sleep Guard</t>
+        </is>
+      </c>
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>A bedtime moment when the tag is tapped</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="inlineStr">
+        <is>
+          <t>Arming locks every blocked app until morning - the most consequential action in the app, and previously the most invisible: the NFC sheet closed and a card quietly changed state. The screen now goes to night, a crescent rises, and the copy states what happened and what is waiting in the morning. A room going dark rather than a celebration. Auto-dismisses after ~4s, any tap skips it, and Reduce Motion collapses it to a short fade. Built on RN Animated to match Anim.jsx, all on useNativeDriver so it does not contend with the JS thread while the shield is applied.</t>
+        </is>
+      </c>
+      <c r="G112" s="16" t="inlineStr">
+        <is>
+          <t>1.1.7</t>
+        </is>
+      </c>
+      <c r="H112" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H109"/>
+  <autoFilter ref="A1:H112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(release): build 123 for the 1.1.7 submission, changelog updated
Bumped CURRENT_PROJECT_VERSION 122 -> 123. Build 122 was cut at bea5e5d and
predates both the deep-link fix and the action plan, so it could not ship as
1.1.7 anyway; reusing its number would also be the duplicate version+build
pair that ITMS-90062 rejects.

MARKETING_VERSION, app.json and package.json all stay at 1.1.7, and
Info.plist keeps both keys variable-driven.

Changelog gains the two rows this build adds: the cold-launch deep-link fix
and the action plan. Per CLAUDE.md that belongs in the same commit as the
bump.

Both were verified on device before this bump — a genuine cold launch from a
Supabase email link lands signed in, and applying a plan installs its blocked
hours without dropping windows the user already had. Release build against
the iOS 27 SDK: BUILD SUCCEEDED.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E112)</f>
+        <f>COUNTA(Changes!E2:E114)</f>
         <v/>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$112,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$114,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$112,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$114,G8)</f>
         <v/>
       </c>
     </row>
@@ -686,16 +686,16 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$112,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$114,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Add Task</t>
+          <t>Action Plan</t>
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$112,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$114,G9)</f>
         <v/>
       </c>
     </row>
@@ -715,16 +715,16 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$112,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$114,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Auth</t>
+          <t>Add Task</t>
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$112,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$114,G10)</f>
         <v/>
       </c>
     </row>
@@ -744,16 +744,16 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$112,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$114,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Auth / Sync</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$112,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$114,G11)</f>
         <v/>
       </c>
     </row>
@@ -773,16 +773,16 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$112,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$114,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Auth / Sync</t>
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$112,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$114,G12)</f>
         <v/>
       </c>
     </row>
@@ -802,16 +802,16 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$112,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$114,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D13)</f>
         <v/>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="H13" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$112,G13)</f>
+        <f>COUNTIF(Changes!$G$2:$G$114,G13)</f>
         <v/>
       </c>
     </row>
@@ -831,335 +831,346 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$112,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$114,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>CI/CD</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>CI/CD</t>
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Challenges</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Dependencies</t>
+          <t>Challenges</t>
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Discoverability</t>
+          <t>Dependencies</t>
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Drift In</t>
+          <t>Discoverability</t>
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Drift In</t>
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Interaction</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Interaction</t>
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Scaling</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Screen Time</t>
+          <t>Scaling</t>
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Screen Time</t>
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Siri</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Sleep Guard</t>
+          <t>Siri</t>
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Tasks</t>
+          <t>Sleep Guard</t>
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Tasks</t>
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Tour</t>
+          <t>Theme</t>
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Tour</t>
         </is>
       </c>
       <c r="E39" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D39)</f>
+        <f>COUNTIF(Changes!$D$2:$D$114,D39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="D40" s="7" t="inlineStr">
         <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E40" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$114,D40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="D41" s="7" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="E40" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$112,D40)</f>
+      <c r="E41" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$114,D41)</f>
         <v/>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>• 1.1.4 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
+          <t>• 1.1.4 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
+          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
         <is>
           <t>• Counts on this sheet are formulas over the Changes tab — they update if you edit, add or delete rows there.</t>
         </is>
@@ -1176,7 +1187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5885,8 +5896,92 @@
         </is>
       </c>
     </row>
+    <row r="113" ht="40" customHeight="1">
+      <c r="A113" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B113" s="16" t="inlineStr">
+        <is>
+          <t>8f645ab</t>
+        </is>
+      </c>
+      <c r="C113" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D113" s="15" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Cold launch from an email link silently did nothing</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="inlineStr">
+        <is>
+          <t>Live in 1.1.6. Tap a Supabase verification link while Drift was backgrounded and it worked; tap it after iOS had reclaimed the app and nothing happened - same user, same link, which is why it read as flaky rather than broken. Under the scene lifecycle both routes to JS are shut at willConnectTo: Linking.getInitialURL() reads only bridge.launchOptions[...URLKey] (RCTLinkingManager.mm:157) and UIKit never populates that key for a scene-based app, while RCTLinkingManager.application(_:open:) merely posts RCTOpenURLNotification, which nothing is listening for before the bundle runs. SceneDelegate forwarded immediately and therefore hit neither. The URL is now held and replayed on RCTContentDidAppearNotification - posted by the Fabric root view once React mounts - plus 0.4s for the gap before Drift.jsx registers its listener, with a 6s timer backing that up in case content appeared before the scene finished connecting. Universal links had the same hole. Because replay makes redelivery routine, the drift://add-friend handler gained the dedupe guard the auth handler already had, claiming the URL BEFORE its first await so two deliveries in one tick cannot both send a friend request. Verified on device: cold-launch email link opens signed in.</t>
+        </is>
+      </c>
+      <c r="G113" s="16" t="inlineStr">
+        <is>
+          <t>1.1.7</t>
+        </is>
+      </c>
+      <c r="H113" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="40" customHeight="1">
+      <c r="A114" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B114" s="16" t="inlineStr">
+        <is>
+          <t>426c33e</t>
+        </is>
+      </c>
+      <c r="C114" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D114" s="15" t="inlineStr">
+        <is>
+          <t>Action Plan</t>
+        </is>
+      </c>
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Build a screen-time plan from a target, a bedtime and a baseline</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="inlineStr">
+        <is>
+          <t>Requested for the JHU pilot: somewhere in the app to build a concrete plan rather than a vague intention. Five answers - typical daily minutes on blocked apps, the target, phone-down time, hardest stretch of the day, what they will do instead - and Drift derives the daily task minutes needed to fund the target, the blocked-hours windows behind it, and the weekly and yearly totals. Deliberately NOT an AI call, unlike every other judgement in the app: a plan someone commits to should be arithmetic they can check, it has to open instantly and work offline, and the same answers must always give the same plan or revising becomes a slot machine. The figure that does the work is the exchange rate - capReward caps rewards at half a task's length, so an hour of scrolling costs two hours of real work. The baseline is self-reported, seeded from today's actual spend, because Apple does not expose Screen Time totals to apps and Drift only knows the minutes it has itself unlocked. Applying MERGES windows into existing blocked hours, matched by id, so re-applying replaces only what the plan created and never drops a window the user set themselves; it also moves the sleep-guard reminder to the phone-down time so the two do not make different promises.</t>
+        </is>
+      </c>
+      <c r="G114" s="16" t="inlineStr">
+        <is>
+          <t>1.1.7</t>
+        </is>
+      </c>
+      <c r="H114" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H112"/>
+  <autoFilter ref="A1:H114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>